<commit_message>
docs : README complet et détaillé
</commit_message>
<xml_diff>
--- a/data/bitcoin.xlsx
+++ b/data/bitcoin.xlsx
@@ -431,311 +431,311 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>15/03/2026</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>61224.44859889374</v>
+        <v>62125.09860849066</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>61878.46175041084</v>
+        <v>63566.1476935859</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62125.09860849066</v>
+        <v>65097.76898262306</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>63566.1476935859</v>
+        <v>64056.15970452876</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>65097.76898262306</v>
+        <v>62144.8037717527</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>20/03/2026</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64056.15970452876</v>
+        <v>60360.61937565861</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>62144.8037717527</v>
+        <v>60971.57878434094</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>60360.61937565861</v>
+        <v>59316.98301318112</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>60971.57878434094</v>
+        <v>58693.95936280688</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>22/03/2026</t>
+          <t>24/03/2026</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>59316.98301318112</v>
+        <v>61076.29831355873</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>25/03/2026</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>58693.95936280688</v>
+        <v>60727.03501227319</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>24/03/2026</t>
+          <t>26/03/2026</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>61076.29831355873</v>
+        <v>61681.08720807594</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>25/03/2026</t>
+          <t>27/03/2026</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>60727.03501227319</v>
+        <v>59635.56440104286</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>26/03/2026</t>
+          <t>28/03/2026</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>61681.08720807594</v>
+        <v>57448.1264426916</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>59635.56440104286</v>
+        <v>57453.14310318966</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>28/03/2026</t>
+          <t>30/03/2026</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>57448.1264426916</v>
+        <v>57411.88733030794</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>57453.14310318966</v>
+        <v>58228.466524081</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>30/03/2026</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>57411.88733030794</v>
+        <v>58984.02933583486</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>58228.466524081</v>
+        <v>58744.37724340737</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>58984.02933583486</v>
+        <v>57957.01182390806</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>58744.37724340737</v>
+        <v>58099.83641408951</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>57957.01182390806</v>
+        <v>58421.30009140765</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>58099.83641408951</v>
+        <v>59937.86767947226</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>58421.30009140765</v>
+        <v>59667.69146335397</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>59937.86767947226</v>
+        <v>61599.11225532703</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>59667.69146335397</v>
+        <v>60999.39280440142</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>61599.11225532703</v>
+        <v>61390.1848793943</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>60999.39280440142</v>
+        <v>62207.70134395084</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>61390.1848793943</v>
+        <v>62298.09108821939</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>62207.70134395084</v>
+        <v>60611.0820347258</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>62627.67213599091</v>
+        <v>62174.97545972216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>